<commit_message>
Enhance application with real-time autocomplete functionality for data selection, improved Excel export formatting with auto-adjusted columns and navy headers, and updated README and PLAN documentation to reflect these changes. Adjusted user interface components for better usability in various sections including Business Intelligence and stock management.
</commit_message>
<xml_diff>
--- a/exports/historial_compras/historial_compras_hasta_2026-07-07.xlsx
+++ b/exports/historial_compras/historial_compras_hasta_2026-07-07.xlsx
@@ -10,9 +10,7 @@
     <sheet name="Info" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Historial" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Historial'!$A$1:$H$12</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -20,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,13 +26,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000B1F3A"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,8 +56,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -125,6 +135,23 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TablaHistorialCompras" displayName="TablaHistorialCompras" ref="A1:H12" headerRowCount="1">
+  <autoFilter ref="A1:H12"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Producto"/>
+    <tableColumn id="2" name="Lote"/>
+    <tableColumn id="3" name="Fecha compra"/>
+    <tableColumn id="4" name="Expiración"/>
+    <tableColumn id="5" name="Cantidad"/>
+    <tableColumn id="6" name="Restante"/>
+    <tableColumn id="7" name="Precio total"/>
+    <tableColumn id="8" name="Proveedor"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -418,14 +445,18 @@
   </sheetPr>
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
@@ -451,7 +482,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>07/07/2026 17:50</t>
+          <t>07/07/2026 17:55</t>
         </is>
       </c>
     </row>
@@ -463,7 +494,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hasta 07/07/2026 — orden: fecha de compra (reciente primero)</t>
+          <t>Hasta 07/07/2026 — orden: nombre (A→Z)</t>
         </is>
       </c>
     </row>
@@ -490,44 +521,54 @@
   </sheetPr>
   <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Lote</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Fecha compra</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Expiración</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Restante</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Precio total</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Proveedor</t>
         </is>
@@ -536,228 +577,228 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Croissant</t>
+          <t>Café molido</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>l11</t>
+          <t>l07</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>07/07/2026</t>
+          <t>22/06/2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10,00 €</t>
+          <t>22,00 €</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>bimbo</t>
+          <t>Cafés Origen</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fruta fresca</t>
+          <t>Croissant</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>l09</t>
+          <t>l01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11/07/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="F3" t="n">
-        <v>2.1</v>
+        <v>42</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>12,00 €</t>
+          <t>18,00 €</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Frutas del Mercado</t>
+          <t>Panadería Sol</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Zumo de naranja</t>
+          <t>Croissant</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>l06</t>
+          <t>l11</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>05/07/2026</t>
+          <t>07/07/2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>12/07/2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>15,00 €</t>
+          <t>10,00 €</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Cítricos Valle</t>
+          <t>bimbo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pan de molde</t>
+          <t>Fruta fresca</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>l02</t>
+          <t>l09</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>04/07/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>14/07/2026</t>
+          <t>11/07/2026</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
-        <v>8</v>
+        <v>2.1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4,50 €</t>
+          <t>12,00 €</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Bimbo</t>
+          <t>Frutas del Mercado</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Yogur natural</t>
+          <t>Huevos</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>l05</t>
+          <t>l10</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>03/07/2026</t>
+          <t>30/06/2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>09/07/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="F6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>12,00 €</t>
+          <t>6,00 €</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Danone</t>
+          <t>Granja Local</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Croissant</t>
+          <t>Jamón serrano</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>l01</t>
+          <t>l03</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>21/07/2026</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>60</v>
+        <v>2.5</v>
       </c>
       <c r="F7" t="n">
-        <v>42</v>
+        <v>1.2</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>18,00 €</t>
+          <t>45,00 €</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Panadería Sol</t>
+          <t>Embutidos Norte</t>
         </is>
       </c>
     </row>
@@ -802,38 +843,38 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Huevos</t>
+          <t>Pan de molde</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>l10</t>
+          <t>l02</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>30/06/2026</t>
+          <t>04/07/2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>14/07/2026</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>6,00 €</t>
+          <t>4,50 €</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Granja Local</t>
+          <t>Bimbo</t>
         </is>
       </c>
     </row>
@@ -878,81 +919,83 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jamón serrano</t>
+          <t>Yogur natural</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>l03</t>
+          <t>l05</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>27/06/2026</t>
+          <t>03/07/2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>21/07/2026</t>
+          <t>09/07/2026</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2.5</v>
+        <v>48</v>
       </c>
       <c r="F11" t="n">
-        <v>1.2</v>
+        <v>10</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>45,00 €</t>
+          <t>12,00 €</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Embutidos Norte</t>
+          <t>Danone</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Café molido</t>
+          <t>Zumo de naranja</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>l07</t>
+          <t>l06</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>22/06/2026</t>
+          <t>05/07/2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>12/07/2026</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1</v>
+        <v>4.5</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>22,00 €</t>
+          <t>15,00 €</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Cafés Origen</t>
+          <t>Cítricos Valle</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>